<commit_message>
Agregada página de accesos_rapidos
</commit_message>
<xml_diff>
--- a/Reporte_Tareas_2026-02-24.xlsx
+++ b/Reporte_Tareas_2026-02-24.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3329,6 +3329,111 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADGG040PO </t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>id=298 alumna que no puede acceder</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>SSCE002PO</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>id=276 alumno que no puede acceder</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>CEC</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Cerrada su cuenta Víctor Bueso Martínez</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3340,15 +3445,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3389,6 +3494,111 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADGG040PO </t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>id=298 alumna que no puede acceder</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>SSCE002PO</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>id=276 alumno que no puede acceder</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fevecta 2026 incidencia</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>fevecta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CEC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Cerrada su cuenta Víctor Bueso Martínez</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>